<commit_message>
customer_service(Feat): refine prompt engineering, optimize tool invocation logic, and add CLI
</commit_message>
<xml_diff>
--- a/customer_service/knowledge_base/knowledge_base_0.xlsx
+++ b/customer_service/knowledge_base/knowledge_base_0.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3002" uniqueCount="2483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3006" uniqueCount="2487">
   <si>
     <t>Query</t>
   </si>
@@ -1533,6 +1533,18 @@
   </si>
   <si>
     <t>why is msg unhealthy</t>
+  </si>
+  <si>
+    <t>小米技术发布会在几号，发布了什么</t>
+  </si>
+  <si>
+    <t>小米技术发布会的具体时间是2025年5月22日，由雷军主持，主要推出了包括自研手机SoC芯片，小米15S Pro还有首款纯电SUV Yu7等</t>
+  </si>
+  <si>
+    <t>切尔西足球俱乐部是否赢得欧协联，对手是谁</t>
+  </si>
+  <si>
+    <t>切尔西在北京时间2025年5月29日凌晨4：1战胜皇家贝蒂斯获得欧协联冠军，并且成为首支欧战大满贯俱乐部</t>
   </si>
   <si>
     <t>爬行垫什么材质的好</t>
@@ -7488,14 +7500,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7968,13 +7973,16 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -7983,118 +7991,115 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -8102,7 +8107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8628,7 +8633,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1501"/>
+  <dimension ref="A1:B1503"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -14812,23 +14817,23 @@
         <v>1044</v>
       </c>
       <c r="B773" s="1" t="s">
-        <v>979</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="774" spans="1:2">
       <c r="A774" s="1" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="B774" s="1" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="775" spans="1:2">
       <c r="A775" s="1" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B775" s="1" t="s">
-        <v>1048</v>
+        <v>983</v>
       </c>
     </row>
     <row r="776" spans="1:2">
@@ -15596,23 +15601,23 @@
         <v>1239</v>
       </c>
       <c r="B871" s="1" t="s">
-        <v>1162</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="872" spans="1:2">
       <c r="A872" s="1" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="B872" s="1" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="873" spans="1:2">
       <c r="A873" s="1" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="B873" s="1" t="s">
-        <v>1243</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="874" spans="1:2">
@@ -15740,23 +15745,23 @@
         <v>1274</v>
       </c>
       <c r="B889" s="1" t="s">
-        <v>1180</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="890" spans="1:2">
       <c r="A890" s="1" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="B890" s="1" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="891" spans="1:2">
       <c r="A891" s="1" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="B891" s="1" t="s">
-        <v>1278</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="892" spans="1:2">
@@ -16468,23 +16473,23 @@
         <v>1455</v>
       </c>
       <c r="B980" s="1" t="s">
-        <v>1436</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="981" spans="1:2">
       <c r="A981" s="1" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="B981" s="1" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="982" spans="1:2">
       <c r="A982" s="1" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="B982" s="1" t="s">
-        <v>1459</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="983" spans="1:2">
@@ -16508,23 +16513,23 @@
         <v>1464</v>
       </c>
       <c r="B985" s="1" t="s">
-        <v>707</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="986" spans="1:2">
       <c r="A986" s="1" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="B986" s="1" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="987" spans="1:2">
       <c r="A987" s="1" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="B987" s="1" t="s">
-        <v>1468</v>
+        <v>711</v>
       </c>
     </row>
     <row r="988" spans="1:2">
@@ -16881,23 +16886,23 @@
     </row>
     <row r="1032" spans="1:2">
       <c r="A1032" s="1" t="s">
-        <v>1545</v>
+        <v>1557</v>
       </c>
       <c r="B1032" s="1" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="1033" spans="1:2">
       <c r="A1033" s="1" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="B1033" s="1" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="1034" spans="1:2">
       <c r="A1034" s="1" t="s">
-        <v>1560</v>
+        <v>1549</v>
       </c>
       <c r="B1034" s="1" t="s">
         <v>1561</v>
@@ -17604,23 +17609,23 @@
         <v>1736</v>
       </c>
       <c r="B1122" s="1" t="s">
-        <v>1731</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="1123" spans="1:2">
       <c r="A1123" s="1" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="B1123" s="1" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="1124" spans="1:2">
       <c r="A1124" s="1" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="B1124" s="1" t="s">
-        <v>1740</v>
+        <v>1735</v>
       </c>
     </row>
     <row r="1125" spans="1:2">
@@ -18356,23 +18361,23 @@
         <v>1923</v>
       </c>
       <c r="B1216" s="1" t="s">
-        <v>1705</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="1217" spans="1:2">
       <c r="A1217" s="1" t="s">
-        <v>1924</v>
+        <v>1925</v>
       </c>
       <c r="B1217" s="1" t="s">
-        <v>1925</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="1218" spans="1:2">
       <c r="A1218" s="1" t="s">
-        <v>1926</v>
+        <v>1927</v>
       </c>
       <c r="B1218" s="1" t="s">
-        <v>1927</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="1219" spans="1:2">
@@ -18497,23 +18502,23 @@
     </row>
     <row r="1234" spans="1:2">
       <c r="A1234" s="1" t="s">
-        <v>1736</v>
+        <v>1958</v>
       </c>
       <c r="B1234" s="1" t="s">
-        <v>1958</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="1235" spans="1:2">
       <c r="A1235" s="1" t="s">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="B1235" s="1" t="s">
-        <v>1960</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="1236" spans="1:2">
       <c r="A1236" s="1" t="s">
-        <v>1961</v>
+        <v>1740</v>
       </c>
       <c r="B1236" s="1" t="s">
         <v>1962</v>
@@ -18540,23 +18545,23 @@
         <v>1967</v>
       </c>
       <c r="B1239" s="1" t="s">
-        <v>1962</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="1240" spans="1:2">
       <c r="A1240" s="1" t="s">
-        <v>1968</v>
+        <v>1969</v>
       </c>
       <c r="B1240" s="1" t="s">
-        <v>1969</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="1241" spans="1:2">
       <c r="A1241" s="1" t="s">
-        <v>1970</v>
+        <v>1971</v>
       </c>
       <c r="B1241" s="1" t="s">
-        <v>1971</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="1242" spans="1:2">
@@ -18572,23 +18577,23 @@
         <v>1974</v>
       </c>
       <c r="B1243" s="1" t="s">
-        <v>1958</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="1244" spans="1:2">
       <c r="A1244" s="1" t="s">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="B1244" s="1" t="s">
-        <v>1976</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="1245" spans="1:2">
       <c r="A1245" s="1" t="s">
-        <v>1977</v>
+        <v>1978</v>
       </c>
       <c r="B1245" s="1" t="s">
-        <v>1978</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="1246" spans="1:2">
@@ -18841,26 +18846,26 @@
     </row>
     <row r="1277" spans="1:2">
       <c r="A1277" s="1" t="s">
-        <v>2037</v>
+        <v>2041</v>
       </c>
       <c r="B1277" s="1" t="s">
-        <v>2038</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="1278" spans="1:2">
       <c r="A1278" s="1" t="s">
-        <v>2041</v>
+        <v>2043</v>
       </c>
       <c r="B1278" s="1" t="s">
-        <v>2042</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="1279" spans="1:2">
       <c r="A1279" s="1" t="s">
-        <v>2043</v>
+        <v>2041</v>
       </c>
       <c r="B1279" s="1" t="s">
-        <v>2044</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="1280" spans="1:2">
@@ -19841,34 +19846,34 @@
     </row>
     <row r="1402" spans="1:2">
       <c r="A1402" s="1" t="s">
-        <v>1736</v>
+        <v>2289</v>
       </c>
       <c r="B1402" s="1" t="s">
-        <v>2289</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="1403" spans="1:2">
       <c r="A1403" s="1" t="s">
-        <v>2290</v>
+        <v>2291</v>
       </c>
       <c r="B1403" s="1" t="s">
-        <v>2140</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="1404" spans="1:2">
       <c r="A1404" s="1" t="s">
-        <v>2291</v>
+        <v>1740</v>
       </c>
       <c r="B1404" s="1" t="s">
-        <v>2292</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="1405" spans="1:2">
       <c r="A1405" s="1" t="s">
-        <v>2293</v>
+        <v>2294</v>
       </c>
       <c r="B1405" s="1" t="s">
-        <v>2294</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="1406" spans="1:2">
@@ -19948,23 +19953,23 @@
         <v>2313</v>
       </c>
       <c r="B1415" s="1" t="s">
-        <v>2292</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="1416" spans="1:2">
       <c r="A1416" s="1" t="s">
-        <v>2314</v>
+        <v>2315</v>
       </c>
       <c r="B1416" s="1" t="s">
-        <v>2315</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="1417" spans="1:2">
       <c r="A1417" s="1" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="B1417" s="1" t="s">
-        <v>2317</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="1418" spans="1:2">
@@ -19996,23 +20001,23 @@
         <v>2324</v>
       </c>
       <c r="B1421" s="1" t="s">
-        <v>2292</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="1422" spans="1:2">
       <c r="A1422" s="1" t="s">
-        <v>2325</v>
+        <v>2326</v>
       </c>
       <c r="B1422" s="1" t="s">
-        <v>2326</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="1423" spans="1:2">
       <c r="A1423" s="1" t="s">
-        <v>2327</v>
+        <v>2328</v>
       </c>
       <c r="B1423" s="1" t="s">
-        <v>2328</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="1424" spans="1:2">
@@ -20100,31 +20105,31 @@
         <v>2349</v>
       </c>
       <c r="B1434" s="1" t="s">
-        <v>2292</v>
+        <v>2350</v>
       </c>
     </row>
     <row r="1435" spans="1:2">
       <c r="A1435" s="1" t="s">
-        <v>2350</v>
+        <v>2351</v>
       </c>
       <c r="B1435" s="1" t="s">
-        <v>2332</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="1436" spans="1:2">
       <c r="A1436" s="1" t="s">
-        <v>2351</v>
+        <v>2353</v>
       </c>
       <c r="B1436" s="1" t="s">
-        <v>2352</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="1437" spans="1:2">
       <c r="A1437" s="1" t="s">
-        <v>2353</v>
+        <v>2354</v>
       </c>
       <c r="B1437" s="1" t="s">
-        <v>2354</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="1438" spans="1:2">
@@ -20637,6 +20642,22 @@
       </c>
       <c r="B1501" s="1" t="s">
         <v>2482</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:2">
+      <c r="A1502" s="1" t="s">
+        <v>2483</v>
+      </c>
+      <c r="B1502" s="1" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:2">
+      <c r="A1503" s="1" t="s">
+        <v>2485</v>
+      </c>
+      <c r="B1503" s="1" t="s">
+        <v>2486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>